<commit_message>
Working Version fo Case 7
</commit_message>
<xml_diff>
--- a/Schlagdifferentialgleichung/Programme/excelDir/CharactExponentenMultiplikatoren_ebeta0dot000_mu0_mu10_Auswahl1.xlsx
+++ b/Schlagdifferentialgleichung/Programme/excelDir/CharactExponentenMultiplikatoren_ebeta0dot000_mu0_mu10_Auswahl1.xlsx
@@ -13,7 +13,94 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="116" uniqueCount="58">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="145" uniqueCount="87">
+  <si>
+    <t>muChar</t>
+  </si>
+  <si>
+    <t>RealCharExp01</t>
+  </si>
+  <si>
+    <t>RealCharExp02</t>
+  </si>
+  <si>
+    <t>RealCharExp03</t>
+  </si>
+  <si>
+    <t>RealCharExp04</t>
+  </si>
+  <si>
+    <t>RealCharExp05</t>
+  </si>
+  <si>
+    <t>RealCharExp06</t>
+  </si>
+  <si>
+    <t>ImagCharExp01</t>
+  </si>
+  <si>
+    <t>ImagCharExp02</t>
+  </si>
+  <si>
+    <t>ImagCharExp03</t>
+  </si>
+  <si>
+    <t>ImagCharExp04</t>
+  </si>
+  <si>
+    <t>ImagCharExp05</t>
+  </si>
+  <si>
+    <t>ImagCharExp06</t>
+  </si>
+  <si>
+    <t>RealCharMult01</t>
+  </si>
+  <si>
+    <t>RealCharMult02</t>
+  </si>
+  <si>
+    <t>RealCharMult03</t>
+  </si>
+  <si>
+    <t>RealCharMult04</t>
+  </si>
+  <si>
+    <t>RealCharMult05</t>
+  </si>
+  <si>
+    <t>RealCharMult06</t>
+  </si>
+  <si>
+    <t>ImagCharMult01</t>
+  </si>
+  <si>
+    <t>ImagCharMult02</t>
+  </si>
+  <si>
+    <t>ImagCharMult03</t>
+  </si>
+  <si>
+    <t>ImagCharMult04</t>
+  </si>
+  <si>
+    <t>ImagCharMult05</t>
+  </si>
+  <si>
+    <t>ImagCharMult06</t>
+  </si>
+  <si>
+    <t>RealCharExp1Corrected</t>
+  </si>
+  <si>
+    <t>ImagCharExp1Corrected</t>
+  </si>
+  <si>
+    <t>RealCharExp2Corrected</t>
+  </si>
+  <si>
+    <t>ImagCharExp2Corrected</t>
+  </si>
   <si>
     <t>muChar</t>
   </si>
@@ -268,91 +355,91 @@
   <sheetData>
     <row r="1">
       <c r="A1" s="0" t="s">
-        <v>29</v>
+        <v>58</v>
       </c>
       <c r="B1" s="0" t="s">
-        <v>30</v>
+        <v>59</v>
       </c>
       <c r="C1" s="0" t="s">
-        <v>31</v>
+        <v>60</v>
       </c>
       <c r="D1" s="0" t="s">
-        <v>32</v>
+        <v>61</v>
       </c>
       <c r="E1" s="0" t="s">
-        <v>33</v>
+        <v>62</v>
       </c>
       <c r="F1" s="0" t="s">
-        <v>34</v>
+        <v>63</v>
       </c>
       <c r="G1" s="0" t="s">
-        <v>35</v>
+        <v>64</v>
       </c>
       <c r="H1" s="0" t="s">
-        <v>36</v>
+        <v>65</v>
       </c>
       <c r="I1" s="0" t="s">
-        <v>37</v>
+        <v>66</v>
       </c>
       <c r="J1" s="0" t="s">
-        <v>38</v>
+        <v>67</v>
       </c>
       <c r="K1" s="0" t="s">
-        <v>39</v>
+        <v>68</v>
       </c>
       <c r="L1" s="0" t="s">
-        <v>40</v>
+        <v>69</v>
       </c>
       <c r="M1" s="0" t="s">
-        <v>41</v>
+        <v>70</v>
       </c>
       <c r="N1" s="0" t="s">
-        <v>42</v>
+        <v>71</v>
       </c>
       <c r="O1" s="0" t="s">
-        <v>43</v>
+        <v>72</v>
       </c>
       <c r="P1" s="0" t="s">
-        <v>44</v>
+        <v>73</v>
       </c>
       <c r="Q1" s="0" t="s">
-        <v>45</v>
+        <v>74</v>
       </c>
       <c r="R1" s="0" t="s">
-        <v>46</v>
+        <v>75</v>
       </c>
       <c r="S1" s="0" t="s">
-        <v>47</v>
+        <v>76</v>
       </c>
       <c r="T1" s="0" t="s">
-        <v>48</v>
+        <v>77</v>
       </c>
       <c r="U1" s="0" t="s">
-        <v>49</v>
+        <v>78</v>
       </c>
       <c r="V1" s="0" t="s">
-        <v>50</v>
+        <v>79</v>
       </c>
       <c r="W1" s="0" t="s">
-        <v>51</v>
+        <v>80</v>
       </c>
       <c r="X1" s="0" t="s">
-        <v>52</v>
+        <v>81</v>
       </c>
       <c r="Y1" s="0" t="s">
-        <v>53</v>
+        <v>82</v>
       </c>
       <c r="Z1" s="0" t="s">
-        <v>54</v>
+        <v>83</v>
       </c>
       <c r="AA1" s="0" t="s">
-        <v>55</v>
+        <v>84</v>
       </c>
       <c r="AB1" s="0" t="s">
-        <v>56</v>
+        <v>85</v>
       </c>
       <c r="AC1" s="0" t="s">
-        <v>57</v>
+        <v>86</v>
       </c>
     </row>
     <row r="2">

</xml_diff>